<commit_message>
Update House PTR data (2026-09-19)
</commit_message>
<xml_diff>
--- a/data/03_verification/House_PTR_Verification_2026.xlsx
+++ b/data/03_verification/House_PTR_Verification_2026.xlsx
@@ -24497,7 +24497,7 @@
       </c>
       <c r="K545" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -67337,7 +67337,7 @@
       </c>
       <c r="K1509" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -74144,7 +74144,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Update House PTR data (2026-10-03)
</commit_message>
<xml_diff>
--- a/data/03_verification/House_PTR_Verification_2026.xlsx
+++ b/data/03_verification/House_PTR_Verification_2026.xlsx
@@ -6578,7 +6578,7 @@
       </c>
       <c r="K142" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -23749,7 +23749,7 @@
       </c>
       <c r="K529" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -69932,7 +69932,7 @@
       </c>
       <c r="K1568" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -76977,7 +76977,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Update House PTR data (2026-10-10)
</commit_message>
<xml_diff>
--- a/data/03_verification/House_PTR_Verification_2026.xlsx
+++ b/data/03_verification/House_PTR_Verification_2026.xlsx
@@ -41501,7 +41501,7 @@
       </c>
       <c r="K925" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>needs_fallback</t>
         </is>
       </c>
     </row>
@@ -78407,7 +78407,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9">
@@ -78417,7 +78417,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -78443,7 +78443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -78810,6 +78810,13 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>9116376</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>